<commit_message>
Corrige calculo caja chica
</commit_message>
<xml_diff>
--- a/Plantilla_Jugadores_Metegol_Areia.xlsx
+++ b/Plantilla_Jugadores_Metegol_Areia.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="38">
   <si>
     <t>Nombre</t>
   </si>
@@ -88,9 +88,6 @@
     <t>Delantero</t>
   </si>
   <si>
-    <t>Tachi Etchegoyen</t>
-  </si>
-  <si>
     <t>Nicolás Gonzales del Cerro</t>
   </si>
   <si>
@@ -122,6 +119,15 @@
   </si>
   <si>
     <t>Tomás De Vicenzi</t>
+  </si>
+  <si>
+    <t>Ignacio Etchegoyen</t>
+  </si>
+  <si>
+    <t>si</t>
+  </si>
+  <si>
+    <t>no</t>
   </si>
 </sst>
 </file>
@@ -547,7 +553,7 @@
         <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -562,7 +568,7 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -583,7 +589,7 @@
         <v>15</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
@@ -606,28 +612,28 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H3">
         <v>0</v>
       </c>
       <c r="I3" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="J3" t="s">
         <v>15</v>
       </c>
       <c r="K3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L3" t="s">
         <v>15</v>
       </c>
       <c r="M3" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="N3">
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
@@ -650,7 +656,7 @@
         <v>0</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4">
         <v>0</v>
@@ -671,7 +677,7 @@
         <v>15</v>
       </c>
       <c r="N4">
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
@@ -679,7 +685,7 @@
         <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -694,7 +700,7 @@
         <v>0</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -715,7 +721,7 @@
         <v>15</v>
       </c>
       <c r="N5">
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
@@ -738,7 +744,7 @@
         <v>0</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6">
         <v>0</v>
@@ -747,10 +753,10 @@
         <v>15</v>
       </c>
       <c r="J6" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="K6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L6" t="s">
         <v>15</v>
@@ -759,7 +765,7 @@
         <v>15</v>
       </c>
       <c r="N6">
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
@@ -767,22 +773,22 @@
         <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C7">
         <v>0</v>
       </c>
       <c r="D7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7">
         <v>0</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -803,7 +809,7 @@
         <v>15</v>
       </c>
       <c r="N7">
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
@@ -826,7 +832,7 @@
         <v>0</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8">
         <v>0</v>
@@ -838,7 +844,7 @@
         <v>15</v>
       </c>
       <c r="K8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L8" t="s">
         <v>15</v>
@@ -847,12 +853,12 @@
         <v>15</v>
       </c>
       <c r="N8">
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="B9" t="s">
         <v>23</v>
@@ -870,7 +876,7 @@
         <v>0</v>
       </c>
       <c r="G9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H9">
         <v>0</v>
@@ -891,12 +897,12 @@
         <v>15</v>
       </c>
       <c r="N9">
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B10" t="s">
         <v>18</v>
@@ -914,7 +920,7 @@
         <v>0</v>
       </c>
       <c r="G10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10">
         <v>0</v>
@@ -935,15 +941,15 @@
         <v>15</v>
       </c>
       <c r="N10">
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -958,7 +964,7 @@
         <v>0</v>
       </c>
       <c r="G11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H11">
         <v>0</v>
@@ -979,12 +985,12 @@
         <v>15</v>
       </c>
       <c r="N11">
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B12" t="s">
         <v>18</v>
@@ -1002,7 +1008,7 @@
         <v>0</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H12">
         <v>0</v>
@@ -1023,12 +1029,12 @@
         <v>15</v>
       </c>
       <c r="N12">
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B13" t="s">
         <v>18</v>
@@ -1046,7 +1052,7 @@
         <v>0</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H13">
         <v>0</v>
@@ -1067,18 +1073,18 @@
         <v>15</v>
       </c>
       <c r="N13">
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B14" t="s">
         <v>18</v>
       </c>
       <c r="C14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14">
         <v>0</v>
@@ -1087,10 +1093,10 @@
         <v>0</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H14">
         <v>0</v>
@@ -1099,10 +1105,10 @@
         <v>15</v>
       </c>
       <c r="J14" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="K14">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L14" t="s">
         <v>15</v>
@@ -1111,15 +1117,15 @@
         <v>15</v>
       </c>
       <c r="N14">
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -1134,13 +1140,13 @@
         <v>0</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H15">
         <v>0</v>
       </c>
       <c r="I15" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="J15" t="s">
         <v>15</v>
@@ -1149,13 +1155,13 @@
         <v>0</v>
       </c>
       <c r="L15" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="M15" t="s">
         <v>15</v>
       </c>
       <c r="N15">
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>